<commit_message>
Fix stale Probability formula in fallback Pipeline templates
</commit_message>
<xml_diff>
--- a/backend/data/templates/pipeline_high.xlsx
+++ b/backend/data/templates/pipeline_high.xlsx
@@ -16,9 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.##%"/>
     <numFmt numFmtId="165" formatCode="&quot;₹&quot;###,##0"/>
+    <numFmt numFmtId="166" formatCode="0.##&quot;%&quot;"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -85,7 +86,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -101,6 +102,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -552,9 +556,8 @@
           <t>Login</t>
         </is>
       </c>
-      <c r="C3" s="3">
-        <f>IF(B3="Login",40%,IF(B3="Sanction",60%,IF(B3="Disbursement",80%,"")))</f>
-        <v/>
+      <c r="C3" s="6" t="n">
+        <v>50</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>

</xml_diff>